<commit_message>
added comps for spark
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E53C541-3E59-45B4-BA30-F500F266ECDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDD431E-FEF2-4514-BA33-21EE1856034A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11580" yWindow="0" windowWidth="16575" windowHeight="15600" activeTab="2" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="241">
   <si>
     <t>Part Number</t>
   </si>
@@ -756,6 +756,15 @@
   </si>
   <si>
     <t>OPAMP</t>
+  </si>
+  <si>
+    <t>AD7804</t>
+  </si>
+  <si>
+    <t>AD7804BRZ</t>
+  </si>
+  <si>
+    <t>AD7804BRZ 16-SOIC (W)</t>
   </si>
 </sst>
 </file>
@@ -1659,8 +1668,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD41208-6905-41A5-8CDA-45891F714057}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="19.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
@@ -1893,6 +1911,29 @@
       </c>
       <c r="H10" t="s">
         <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E11" t="s">
+        <v>238</v>
+      </c>
+      <c r="F11" t="s">
+        <v>190</v>
+      </c>
+      <c r="G11" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
moved comps to specified groups
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDD431E-FEF2-4514-BA33-21EE1856034A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B62F02D-F667-4802-A16C-F06FE3C6FDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="6570" yWindow="2070" windowWidth="21585" windowHeight="11775" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="217">
   <si>
     <t>Part Number</t>
   </si>
@@ -644,36 +644,6 @@
     <t>TPA626</t>
   </si>
   <si>
-    <t>HMC525ALC4</t>
-  </si>
-  <si>
-    <t>LCC-E-24-1</t>
-  </si>
-  <si>
-    <t>HMC525ALC4 LCC E-24-1</t>
-  </si>
-  <si>
-    <t>LCC E-24-1</t>
-  </si>
-  <si>
-    <t>HMC427ALP3E</t>
-  </si>
-  <si>
-    <t>QFN-16</t>
-  </si>
-  <si>
-    <t>HMC427ALP3E QFN-16</t>
-  </si>
-  <si>
-    <t>16-QFN (3X3)</t>
-  </si>
-  <si>
-    <t>HMC902LP3E</t>
-  </si>
-  <si>
-    <t>HMC902LP3E QFN-16</t>
-  </si>
-  <si>
     <t>74ACT74MTC</t>
   </si>
   <si>
@@ -683,12 +653,6 @@
     <t>74ACT74MTC TSSOP-16</t>
   </si>
   <si>
-    <t>74ACT04MTC</t>
-  </si>
-  <si>
-    <t>74ACT04MTC TSSOP-14</t>
-  </si>
-  <si>
     <t>ADG608BR</t>
   </si>
   <si>
@@ -711,42 +675,6 @@
   </si>
   <si>
     <t>TP1961-TR SOT23-5</t>
-  </si>
-  <si>
-    <t>THS4503CDGNR</t>
-  </si>
-  <si>
-    <t>8-MSOP-EP</t>
-  </si>
-  <si>
-    <t>THS4503CDGNR 8-MSOP-EP</t>
-  </si>
-  <si>
-    <t>THS4503</t>
-  </si>
-  <si>
-    <t>HMC407MS8G</t>
-  </si>
-  <si>
-    <t>HFCN-5050+</t>
-  </si>
-  <si>
-    <t>Mini Circuits</t>
-  </si>
-  <si>
-    <t>LFCN-6000D+</t>
-  </si>
-  <si>
-    <t>SKY16601-555LF</t>
-  </si>
-  <si>
-    <t>Skyworks Solutions</t>
-  </si>
-  <si>
-    <t>HMC717ALP3E</t>
-  </si>
-  <si>
-    <t>HMC717ALP3E 16-QFN (3X3)</t>
   </si>
   <si>
     <t>AD8065</t>
@@ -1640,16 +1568,16 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="B6" t="s">
         <v>170</v>
       </c>
       <c r="C6" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="D6" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>93</v>
@@ -1915,19 +1843,19 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>239</v>
+        <v>215</v>
       </c>
       <c r="B11" t="s">
         <v>190</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>240</v>
+        <v>216</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>239</v>
+        <v>215</v>
       </c>
       <c r="E11" t="s">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="F11" t="s">
         <v>190</v>
@@ -2158,8 +2086,16 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6417C9C4-F4DF-4AC8-B50B-4BF5CA8F6EE6}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
@@ -2323,6 +2259,29 @@
       </c>
       <c r="G7" s="3" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>211</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>212</v>
+      </c>
+      <c r="D8" t="s">
+        <v>211</v>
+      </c>
+      <c r="E8" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2332,8 +2291,13 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919936B4-B1A4-46D7-993E-F45D36458108}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="35.28515625" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
@@ -2539,333 +2503,68 @@
         <v>200</v>
       </c>
       <c r="F9" t="s">
+        <v>201</v>
+      </c>
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="G9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>204</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="F10" t="s">
         <v>206</v>
-      </c>
-      <c r="D10" t="s">
-        <v>204</v>
-      </c>
-      <c r="E10" t="s">
-        <v>204</v>
-      </c>
-      <c r="F10" t="s">
-        <v>207</v>
       </c>
       <c r="G10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B11" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B11" t="s">
-        <v>205</v>
-      </c>
-      <c r="C11" t="s">
-        <v>209</v>
-      </c>
-      <c r="D11" t="s">
-        <v>208</v>
-      </c>
-      <c r="E11" t="s">
-        <v>208</v>
+      <c r="D11" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>207</v>
       </c>
       <c r="F11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>210</v>
-      </c>
-      <c r="B12" t="s">
-        <v>211</v>
-      </c>
-      <c r="C12" t="s">
-        <v>212</v>
-      </c>
-      <c r="D12" t="s">
-        <v>210</v>
-      </c>
-      <c r="E12" t="s">
-        <v>210</v>
-      </c>
-      <c r="F12" t="s">
-        <v>211</v>
-      </c>
-      <c r="G12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>213</v>
-      </c>
-      <c r="B13" t="s">
-        <v>159</v>
-      </c>
-      <c r="C13" t="s">
-        <v>214</v>
-      </c>
-      <c r="D13" t="s">
-        <v>213</v>
-      </c>
-      <c r="E13" t="s">
-        <v>213</v>
-      </c>
-      <c r="F13" t="s">
-        <v>211</v>
-      </c>
-      <c r="G13" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B14" t="s">
-        <v>216</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="F14" t="s">
-        <v>218</v>
-      </c>
-      <c r="G14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="B15" t="s">
-        <v>216</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F15" t="s">
-        <v>218</v>
-      </c>
-      <c r="G15" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>221</v>
-      </c>
-      <c r="B16" t="s">
-        <v>170</v>
-      </c>
-      <c r="C16" t="s">
-        <v>222</v>
-      </c>
-      <c r="D16" t="s">
-        <v>221</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F16" t="s">
-        <v>170</v>
-      </c>
-      <c r="G16" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B17" t="s">
-        <v>224</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="G18" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" t="s">
-        <v>228</v>
-      </c>
-      <c r="B19" t="s">
-        <v>228</v>
-      </c>
-      <c r="C19" t="s">
-        <v>228</v>
-      </c>
-      <c r="D19" t="s">
-        <v>228</v>
-      </c>
-      <c r="E19" t="s">
-        <v>228</v>
-      </c>
-      <c r="F19" t="s">
-        <v>228</v>
-      </c>
-      <c r="G19" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" t="s">
-        <v>230</v>
-      </c>
-      <c r="B20" t="s">
-        <v>230</v>
-      </c>
-      <c r="C20" t="s">
-        <v>230</v>
-      </c>
-      <c r="D20" t="s">
-        <v>230</v>
-      </c>
-      <c r="E20" t="s">
-        <v>230</v>
-      </c>
-      <c r="F20" t="s">
-        <v>230</v>
-      </c>
-      <c r="G20" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
-        <v>231</v>
-      </c>
-      <c r="B21" t="s">
-        <v>231</v>
-      </c>
-      <c r="C21" t="s">
-        <v>231</v>
-      </c>
-      <c r="D21" t="s">
-        <v>231</v>
-      </c>
-      <c r="E21" t="s">
-        <v>231</v>
-      </c>
-      <c r="F21" t="s">
-        <v>231</v>
-      </c>
-      <c r="G21" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="B22" t="s">
-        <v>207</v>
-      </c>
-      <c r="C22" t="s">
-        <v>234</v>
-      </c>
-      <c r="D22" t="s">
-        <v>233</v>
-      </c>
-      <c r="E22" t="s">
-        <v>233</v>
-      </c>
-      <c r="F22" t="s">
-        <v>207</v>
-      </c>
-      <c r="G22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" t="s">
-        <v>235</v>
-      </c>
-      <c r="B23" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" t="s">
-        <v>236</v>
-      </c>
-      <c r="D23" t="s">
-        <v>235</v>
-      </c>
-      <c r="E23" t="s">
-        <v>237</v>
-      </c>
-      <c r="F23" t="s">
-        <v>39</v>
-      </c>
-      <c r="G23" t="s">
-        <v>25</v>
-      </c>
+    <row r="18" spans="1:6">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added opamp and 0201
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git\elem_altium_db2\library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B62F02D-F667-4802-A16C-F06FE3C6FDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142D6991-3820-494D-9D9E-4C896F3DD5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6570" yWindow="2070" windowWidth="21585" windowHeight="11775" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="218">
   <si>
     <t>Part Number</t>
   </si>
@@ -693,6 +693,9 @@
   </si>
   <si>
     <t>AD7804BRZ 16-SOIC (W)</t>
+  </si>
+  <si>
+    <t>ADA4851-2YRMZ-RL7</t>
   </si>
 </sst>
 </file>
@@ -2086,13 +2089,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6417C9C4-F4DF-4AC8-B50B-4BF5CA8F6EE6}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
     <col min="2" max="2" width="13.140625" customWidth="1"/>
     <col min="3" max="3" width="24.5703125" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" customWidth="1"/>
   </cols>
@@ -2281,6 +2284,29 @@
         <v>39</v>
       </c>
       <c r="G8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>217</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>217</v>
+      </c>
+      <c r="D9" t="s">
+        <v>217</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="F9" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added LSM6 and 50A-15BX
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142D6991-3820-494D-9D9E-4C896F3DD5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB1340F-5856-4535-8E8A-ACE651AE3BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="220">
   <si>
     <t>Part Number</t>
   </si>
@@ -696,6 +696,12 @@
   </si>
   <si>
     <t>ADA4851-2YRMZ-RL7</t>
+  </si>
+  <si>
+    <t>LSM6DS3TR-C</t>
+  </si>
+  <si>
+    <t>14-LGA</t>
   </si>
 </sst>
 </file>
@@ -2599,8 +2605,17 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF27F01-F832-4718-B945-C43E22A8DD17}">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27.42578125" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="3" max="3" width="25.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="29.42578125" customWidth="1"/>
+    <col min="7" max="7" width="21.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
@@ -2781,6 +2796,26 @@
         <v>146</v>
       </c>
     </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C8" t="s">
+        <v>218</v>
+      </c>
+      <c r="D8" t="s">
+        <v>218</v>
+      </c>
+      <c r="E8" t="s">
+        <v>218</v>
+      </c>
+      <c r="F8" t="s">
+        <v>219</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
there's been a lot
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69715850-051B-4AF7-A386-7A2B8E55A680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514499DB-21BF-4333-AAED-710BDF11CF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="224">
   <si>
     <t>Part Number</t>
   </si>
@@ -711,6 +711,9 @@
   </si>
   <si>
     <t>74HC4052D</t>
+  </si>
+  <si>
+    <t>ADA4851-2YRMZ-RL7 8-MSOP</t>
   </si>
 </sst>
 </file>
@@ -2314,10 +2317,10 @@
         <v>217</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C9" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="D9" t="s">
         <v>217</v>
@@ -2326,7 +2329,7 @@
         <v>157</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="G9" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
added STB24NF10 (TO-263) & 1EDB8275F
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE768480-5756-42BC-9E28-060996D5FEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1606DDF2-A0B4-4354-8D85-EC6B8E8405B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="234">
   <si>
     <t>Part Number</t>
   </si>
@@ -735,6 +735,15 @@
   </si>
   <si>
     <t>INA125PA 16-SOIC</t>
+  </si>
+  <si>
+    <t>1EDB8275F</t>
+  </si>
+  <si>
+    <t>1EDBx275F</t>
+  </si>
+  <si>
+    <t>Infineon</t>
   </si>
 </sst>
 </file>
@@ -2735,6 +2744,29 @@
         <v>64</v>
       </c>
     </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>231</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>231</v>
+      </c>
+      <c r="D13" t="s">
+        <v>231</v>
+      </c>
+      <c r="E13" t="s">
+        <v>232</v>
+      </c>
+      <c r="F13" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" t="s">
+        <v>233</v>
+      </c>
+    </row>
     <row r="18" spans="1:6">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>

</xml_diff>

<commit_message>
misc rf and pwr for bakaev
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1606DDF2-A0B4-4354-8D85-EC6B8E8405B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A7E849-3459-4E11-905D-53A053AA6DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="239">
   <si>
     <t>Part Number</t>
   </si>
@@ -744,6 +744,21 @@
   </si>
   <si>
     <t>Infineon</t>
+  </si>
+  <si>
+    <t>ADA4891-1ARZ</t>
+  </si>
+  <si>
+    <t>ADA4891-1ARZ 8-SOIC</t>
+  </si>
+  <si>
+    <t>ADG1201</t>
+  </si>
+  <si>
+    <t>ADG1201BRJZ-R2</t>
+  </si>
+  <si>
+    <t>ADG1201BRJZ-R2 SOT23-6</t>
   </si>
 </sst>
 </file>
@@ -2200,7 +2215,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6417C9C4-F4DF-4AC8-B50B-4BF5CA8F6EE6}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.42578125" customWidth="1"/>
@@ -2443,6 +2458,29 @@
       </c>
       <c r="G10" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>234</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" t="s">
+        <v>234</v>
+      </c>
+      <c r="E11" t="s">
+        <v>211</v>
+      </c>
+      <c r="F11" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -2607,7 +2645,7 @@
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>192</v>
       </c>
       <c r="B7" t="s">
@@ -2630,7 +2668,7 @@
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>195</v>
       </c>
       <c r="B8" t="s">
@@ -2676,7 +2714,7 @@
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>201</v>
       </c>
       <c r="B10" t="s">
@@ -2699,7 +2737,7 @@
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>205</v>
       </c>
       <c r="B11" t="s">
@@ -2722,7 +2760,7 @@
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="4" t="s">
+      <c r="A12" t="s">
         <v>220</v>
       </c>
       <c r="B12" t="s">
@@ -2767,8 +2805,30 @@
         <v>233</v>
       </c>
     </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>237</v>
+      </c>
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>238</v>
+      </c>
+      <c r="D14" t="s">
+        <v>237</v>
+      </c>
+      <c r="E14" t="s">
+        <v>236</v>
+      </c>
+      <c r="F14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+    </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -2780,6 +2840,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fixed ru comps, added pwr and res
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F65A2326-4EAC-4972-AA10-E4ACB1FA40EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6A67FD-48DB-4EDC-B5B9-91966EBB02B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="257">
   <si>
     <t>Part Number</t>
   </si>
@@ -801,6 +801,18 @@
   </si>
   <si>
     <t>1401СА1 14-DIP</t>
+  </si>
+  <si>
+    <t>AD5160</t>
+  </si>
+  <si>
+    <t>SOT23-8</t>
+  </si>
+  <si>
+    <t>AD5160 SOT23-8</t>
+  </si>
+  <si>
+    <t>AD5160BRJ5-RL7</t>
   </si>
 </sst>
 </file>
@@ -2595,7 +2607,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919936B4-B1A4-46D7-993E-F45D36458108}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
@@ -2970,6 +2982,29 @@
       </c>
       <c r="H16" t="s">
         <v>249</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>256</v>
+      </c>
+      <c r="B17" t="s">
+        <v>254</v>
+      </c>
+      <c r="C17" t="s">
+        <v>255</v>
+      </c>
+      <c r="D17" t="s">
+        <v>253</v>
+      </c>
+      <c r="E17" t="s">
+        <v>253</v>
+      </c>
+      <c r="F17" t="s">
+        <v>254</v>
+      </c>
+      <c r="G17" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added 200V dc-dc comps
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB820D01-4EF3-4DF1-A0A8-DE74583D83FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7B49F8-02D0-4BB2-8AB5-12782A318F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="262">
   <si>
     <t>Part Number</t>
   </si>
@@ -749,9 +749,6 @@
     <t>ADA4891-1ARZ</t>
   </si>
   <si>
-    <t>ADA4891-1ARZ 8-SOIC</t>
-  </si>
-  <si>
     <t>ADG1201</t>
   </si>
   <si>
@@ -825,6 +822,12 @@
   </si>
   <si>
     <t>74HC4051PW 16-TSSOP</t>
+  </si>
+  <si>
+    <t>ADA4851-1YRJZ-RL7</t>
+  </si>
+  <si>
+    <t>ADA4891-1ARZ SOT23-6</t>
   </si>
 </sst>
 </file>
@@ -1779,25 +1782,25 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D7" t="s">
+        <v>249</v>
+      </c>
+      <c r="E7" t="s">
+        <v>241</v>
+      </c>
+      <c r="F7" t="s">
+        <v>243</v>
+      </c>
+      <c r="H7" t="s">
         <v>250</v>
-      </c>
-      <c r="E7" t="s">
-        <v>242</v>
-      </c>
-      <c r="F7" t="s">
-        <v>244</v>
-      </c>
-      <c r="H7" t="s">
-        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -2547,19 +2550,19 @@
         <v>234</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>235</v>
+        <v>261</v>
       </c>
       <c r="D11" t="s">
         <v>234</v>
       </c>
       <c r="E11" t="s">
-        <v>211</v>
+        <v>260</v>
       </c>
       <c r="F11" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G11" t="s">
         <v>24</v>
@@ -2567,16 +2570,16 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B12" t="s">
         <v>164</v>
       </c>
       <c r="C12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E12" t="s">
         <v>159</v>
@@ -2590,25 +2593,25 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B13" t="s">
+        <v>243</v>
+      </c>
+      <c r="C13" t="s">
         <v>244</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E13" t="s">
+        <v>242</v>
+      </c>
+      <c r="F13" t="s">
+        <v>243</v>
+      </c>
+      <c r="H13" t="s">
         <v>245</v>
-      </c>
-      <c r="D13" t="s">
-        <v>241</v>
-      </c>
-      <c r="E13" t="s">
-        <v>243</v>
-      </c>
-      <c r="F13" t="s">
-        <v>244</v>
-      </c>
-      <c r="H13" t="s">
-        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -2935,19 +2938,19 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B14" t="s">
         <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E14" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F14" t="s">
         <v>51</v>
@@ -2958,62 +2961,62 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
+        <v>246</v>
+      </c>
+      <c r="C15" t="s">
+        <v>246</v>
+      </c>
+      <c r="D15" t="s">
+        <v>246</v>
+      </c>
+      <c r="E15" t="s">
+        <v>246</v>
+      </c>
+      <c r="F15" t="s">
         <v>247</v>
       </c>
-      <c r="C15" t="s">
-        <v>247</v>
-      </c>
-      <c r="D15" t="s">
-        <v>247</v>
-      </c>
-      <c r="E15" t="s">
-        <v>247</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>248</v>
-      </c>
-      <c r="H15" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
+        <v>247</v>
+      </c>
+      <c r="C16" t="s">
+        <v>247</v>
+      </c>
+      <c r="D16" t="s">
+        <v>247</v>
+      </c>
+      <c r="E16" t="s">
+        <v>247</v>
+      </c>
+      <c r="F16" t="s">
+        <v>247</v>
+      </c>
+      <c r="H16" t="s">
         <v>248</v>
-      </c>
-      <c r="C16" t="s">
-        <v>248</v>
-      </c>
-      <c r="D16" t="s">
-        <v>248</v>
-      </c>
-      <c r="E16" t="s">
-        <v>248</v>
-      </c>
-      <c r="F16" t="s">
-        <v>248</v>
-      </c>
-      <c r="H16" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C17" t="s">
         <v>254</v>
       </c>
-      <c r="C17" t="s">
-        <v>255</v>
-      </c>
       <c r="D17" t="s">
+        <v>252</v>
+      </c>
+      <c r="E17" t="s">
+        <v>252</v>
+      </c>
+      <c r="F17" t="s">
         <v>253</v>
-      </c>
-      <c r="E17" t="s">
-        <v>253</v>
-      </c>
-      <c r="F17" t="s">
-        <v>254</v>
       </c>
       <c r="G17" t="s">
         <v>24</v>
@@ -3021,25 +3024,25 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B18" t="s">
         <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D18" t="s">
+        <v>256</v>
+      </c>
+      <c r="E18" t="s">
         <v>257</v>
-      </c>
-      <c r="E18" t="s">
-        <v>258</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
       </c>
       <c r="G18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HUGE library update: - fixed formatting of all sch components - fixed wrong sch components and changed to unified view - changed main font to GOST instead of GOST type A - added and fixed position of .Designator in pcb components - fixed size field of most ic in tables (correct is SOIC-8, not 8-SOIC, but in pcb library it must be named 8-SOIC due to correct sorting) - fixed value field of all discrete components
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/garou/Documents/work/elem_altium_db2/library/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA142C6-AEB0-470B-A9E2-F78818342584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C21A26-32BD-F649-815F-A8C77299F43F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="8" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="277">
   <si>
     <t>Part Number</t>
   </si>
@@ -191,9 +191,6 @@
     <t>64-LQFP</t>
   </si>
   <si>
-    <t>ADS1675IPAG 64-LQFP</t>
-  </si>
-  <si>
     <t>SN74AVC1T45DBVR</t>
   </si>
   <si>
@@ -203,9 +200,6 @@
     <t>SN74AVC1T45DBVR SOT23-6</t>
   </si>
   <si>
-    <t>74AVC1T45</t>
-  </si>
-  <si>
     <t>SN74LVC2T45DCUR</t>
   </si>
   <si>
@@ -215,9 +209,6 @@
     <t>SN74LVC2T45DCUR VSSOP-8</t>
   </si>
   <si>
-    <t>74AVC2T45</t>
-  </si>
-  <si>
     <t>8-VSSOP</t>
   </si>
   <si>
@@ -401,9 +392,6 @@
     <t>8-MSOP</t>
   </si>
   <si>
-    <t>TPC116S1 8-MSOP</t>
-  </si>
-  <si>
     <t>3PEAK</t>
   </si>
   <si>
@@ -452,15 +440,9 @@
     <t>ISL29033IROZ-T7</t>
   </si>
   <si>
-    <t>ISL29033IROZ-T7 6-ODFN</t>
-  </si>
-  <si>
     <t>ISL29003IROZ-T7</t>
   </si>
   <si>
-    <t>ISL29003IROZ-T7 6-ODFN</t>
-  </si>
-  <si>
     <t>ISL29003IROZ-T7 (Obsolete)</t>
   </si>
   <si>
@@ -674,9 +656,6 @@
     <t>AD8065</t>
   </si>
   <si>
-    <t>AD8065 8-SOIC</t>
-  </si>
-  <si>
     <t>OPAMP</t>
   </si>
   <si>
@@ -686,9 +665,6 @@
     <t>AD7804BRZ</t>
   </si>
   <si>
-    <t>AD7804BRZ 16-SOIC (W)</t>
-  </si>
-  <si>
     <t>ADA4851-2YRMZ-RL7</t>
   </si>
   <si>
@@ -701,21 +677,12 @@
     <t>74HC4052</t>
   </si>
   <si>
-    <t>74HC4052 16-SOIC</t>
-  </si>
-  <si>
     <t>74HC4052D</t>
   </si>
   <si>
-    <t>ADA4851-2YRMZ-RL7 8-MSOP</t>
-  </si>
-  <si>
     <t>AD9288BSTZ-40</t>
   </si>
   <si>
-    <t>AD9288BSTZ-40 48-LQFP</t>
-  </si>
-  <si>
     <t>AD9288</t>
   </si>
   <si>
@@ -731,12 +698,6 @@
     <t>AD7683</t>
   </si>
   <si>
-    <t>AD7683BRMZ 8-MSOP</t>
-  </si>
-  <si>
-    <t>INA125PA 16-SOIC</t>
-  </si>
-  <si>
     <t>1EDB8275F</t>
   </si>
   <si>
@@ -761,9 +722,6 @@
     <t>ADA4891-4ARZ</t>
   </si>
   <si>
-    <t>ADA4891-4ARZ 14-SOIC</t>
-  </si>
-  <si>
     <t>140УД20А ВК</t>
   </si>
   <si>
@@ -776,9 +734,6 @@
     <t>14-DIP</t>
   </si>
   <si>
-    <t>140УД20А ВК 14-DIP</t>
-  </si>
-  <si>
     <t>АЕЯР.431130.149-03ТУ</t>
   </si>
   <si>
@@ -797,9 +752,6 @@
     <t>АЕЯР.431130.171-14ТУ</t>
   </si>
   <si>
-    <t>1401СА1 14-DIP</t>
-  </si>
-  <si>
     <t>AD5160</t>
   </si>
   <si>
@@ -819,9 +771,6 @@
   </si>
   <si>
     <t>Nexperia</t>
-  </si>
-  <si>
-    <t>74HC4051PW 16-TSSOP</t>
   </si>
   <si>
     <t>ADA4851-1YRJZ-RL7</t>
@@ -846,10 +795,94 @@
     <t>AD8138</t>
   </si>
   <si>
-    <t>AD8138 8-SOIC</t>
-  </si>
-  <si>
     <t>ADA4851-1YRJZ-RL7 SOT23-6</t>
+  </si>
+  <si>
+    <t>74LVC1T45</t>
+  </si>
+  <si>
+    <t>74LVC2T45</t>
+  </si>
+  <si>
+    <t>ADS1675IPAG LQFP-64</t>
+  </si>
+  <si>
+    <t>AD9288BSTZ-40 LQFP-48</t>
+  </si>
+  <si>
+    <t>AD7683BRMZ MSOP-8</t>
+  </si>
+  <si>
+    <t>TPC116S1 MSOP-8</t>
+  </si>
+  <si>
+    <t>AD7804BRZ SOIC-16W</t>
+  </si>
+  <si>
+    <t>MSOP-8</t>
+  </si>
+  <si>
+    <t>LQFP-48</t>
+  </si>
+  <si>
+    <t>LQFP-64</t>
+  </si>
+  <si>
+    <t>DIP-14</t>
+  </si>
+  <si>
+    <t>1401СА1 ММ DIP-14</t>
+  </si>
+  <si>
+    <t>1401СА1</t>
+  </si>
+  <si>
+    <t>AD8065 SOIC-8</t>
+  </si>
+  <si>
+    <t>ADA4851-2YRMZ-RL7 MSOP-8</t>
+  </si>
+  <si>
+    <t>INA125PA SOIC-16</t>
+  </si>
+  <si>
+    <t>ADA4891-4ARZ SOIC-14</t>
+  </si>
+  <si>
+    <t>140УД20А ВК DIP-14</t>
+  </si>
+  <si>
+    <t>AD8138 SOIC-8</t>
+  </si>
+  <si>
+    <t>1EDB8275F SOIC-8</t>
+  </si>
+  <si>
+    <t>74HC4052 SOIC-16</t>
+  </si>
+  <si>
+    <t>AT42QT1010-TSHR SOT23-6</t>
+  </si>
+  <si>
+    <t>AD8400AR1 SOIC-8</t>
+  </si>
+  <si>
+    <t>74HC4051PW TSSOP-16</t>
+  </si>
+  <si>
+    <t>ISL29033IROZ-T7 ODFN-6</t>
+  </si>
+  <si>
+    <t>ISL29003IROZ-T7 ODFN-6</t>
+  </si>
+  <si>
+    <t>LSM6DS3TR-C LGA-14</t>
+  </si>
+  <si>
+    <t>LGA-14</t>
+  </si>
+  <si>
+    <t>IRS-B210ST01-R1 5-SMD</t>
   </si>
 </sst>
 </file>
@@ -917,8 +950,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Accent 3 2" xfId="1" xr:uid="{07D6D35A-A25D-4183-ACA2-756DA14CBAEA}"/>
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -934,9 +967,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office 2013–2022">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -974,7 +1007,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1080,7 +1113,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1222,7 +1255,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1231,15 +1264,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67671D6E-5D55-4C0C-9FE7-A86F937C6875}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.42578125" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" customWidth="1"/>
-    <col min="7" max="7" width="36.42578125" customWidth="1"/>
+    <col min="1" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1273,7 +1302,7 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>256</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
@@ -1296,7 +1325,7 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
@@ -1319,7 +1348,7 @@
         <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
         <v>32</v>
@@ -1342,7 +1371,7 @@
         <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
@@ -1365,7 +1394,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>256</v>
       </c>
       <c r="C6" t="s">
         <v>40</v>
@@ -1411,10 +1440,10 @@
         <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>257</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>49</v>
+        <v>250</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>47</v>
@@ -1431,19 +1460,19 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>256</v>
       </c>
       <c r="C9" t="s">
-        <v>223</v>
+        <v>251</v>
       </c>
       <c r="D9" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="E9" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="F9" t="s">
         <v>23</v>
@@ -1454,22 +1483,22 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="B10" t="s">
-        <v>118</v>
+        <v>255</v>
       </c>
       <c r="C10" t="s">
-        <v>229</v>
+        <v>252</v>
       </c>
       <c r="D10" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="E10" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="F10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G10" t="s">
         <v>24</v>
@@ -1484,7 +1513,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E834B2D-3CFC-49B2-A2B4-67F2231F306F}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
@@ -1514,22 +1548,22 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" t="s">
         <v>50</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>51</v>
       </c>
-      <c r="C2" t="s">
-        <v>52</v>
-      </c>
       <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F2" t="s">
         <v>50</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F2" t="s">
-        <v>51</v>
       </c>
       <c r="G2" t="s">
         <v>30</v>
@@ -1537,22 +1571,22 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
         <v>54</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" t="s">
         <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F3" t="s">
-        <v>58</v>
       </c>
       <c r="G3" t="s">
         <v>30</v>
@@ -1560,94 +1594,94 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" t="s">
+      <c r="F4" t="s">
         <v>60</v>
       </c>
-      <c r="C4" t="s">
+      <c r="G4" t="s">
         <v>61</v>
-      </c>
-      <c r="D4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G4" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" t="s">
         <v>65</v>
       </c>
-      <c r="B5" t="s">
+      <c r="F5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" t="s">
         <v>66</v>
-      </c>
-      <c r="C5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E5" t="s">
-        <v>68</v>
-      </c>
-      <c r="F5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" t="s">
         <v>70</v>
       </c>
-      <c r="B6" t="s">
-        <v>71</v>
-      </c>
-      <c r="C6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" t="s">
-        <v>73</v>
-      </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" t="s">
         <v>55</v>
       </c>
-      <c r="C7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7" t="s">
-        <v>74</v>
-      </c>
-      <c r="E7" t="s">
-        <v>74</v>
-      </c>
-      <c r="F7" t="s">
-        <v>58</v>
-      </c>
       <c r="G7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1658,12 +1692,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE4D8C3D-D832-496B-AB92-259D2AD291EC}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
-    <col min="4" max="5" width="24.7109375" customWidth="1"/>
+    <col min="1" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1694,22 +1727,22 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="F2" t="s">
         <v>78</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F2" t="s">
-        <v>81</v>
       </c>
       <c r="G2" t="s">
         <v>24</v>
@@ -1717,19 +1750,19 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F3" t="s">
         <v>38</v>
@@ -1740,19 +1773,19 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
         <v>38</v>
@@ -1763,71 +1796,71 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E5" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="F5" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E5" t="s">
-        <v>91</v>
-      </c>
-      <c r="F5" t="s">
-        <v>92</v>
-      </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C6" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D6" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F6" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="B7" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="C7" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="D7" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="E7" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="F7" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H7" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -1838,15 +1871,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD41208-6905-41A5-8CDA-45891F714057}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="4" width="23.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" customWidth="1"/>
+    <col min="1" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1877,45 +1906,45 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H2" t="s">
         <v>93</v>
-      </c>
-      <c r="B2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C2" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F2" t="s">
-        <v>94</v>
-      </c>
-      <c r="H2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E3" t="s">
         <v>97</v>
       </c>
-      <c r="B3" t="s">
+      <c r="F3" t="s">
         <v>98</v>
-      </c>
-      <c r="C3" t="s">
-        <v>99</v>
-      </c>
-      <c r="D3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F3" t="s">
-        <v>101</v>
       </c>
       <c r="G3" t="s">
         <v>24</v>
@@ -1923,22 +1952,22 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E4" t="s">
         <v>102</v>
       </c>
-      <c r="B4" t="s">
+      <c r="F4" t="s">
         <v>103</v>
-      </c>
-      <c r="C4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E4" t="s">
-        <v>105</v>
-      </c>
-      <c r="F4" t="s">
-        <v>106</v>
       </c>
       <c r="G4" t="s">
         <v>24</v>
@@ -1946,22 +1975,22 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G5" t="s">
         <v>30</v>
@@ -1969,22 +1998,22 @@
     </row>
     <row r="6" spans="1:8" ht="12.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" t="s">
         <v>78</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" t="s">
-        <v>112</v>
-      </c>
-      <c r="F6" t="s">
-        <v>81</v>
       </c>
       <c r="G6" t="s">
         <v>30</v>
@@ -1992,22 +2021,22 @@
     </row>
     <row r="7" spans="1:8" ht="12.75" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F7" t="s">
         <v>78</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E7" t="s">
-        <v>112</v>
-      </c>
-      <c r="F7" t="s">
-        <v>81</v>
       </c>
       <c r="G7" t="s">
         <v>30</v>
@@ -2015,22 +2044,22 @@
     </row>
     <row r="8" spans="1:8" ht="12.75" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F8" t="s">
         <v>78</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F8" t="s">
-        <v>81</v>
       </c>
       <c r="G8" t="s">
         <v>30</v>
@@ -2038,68 +2067,68 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B9" t="s">
-        <v>118</v>
+        <v>255</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>119</v>
+        <v>253</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F9" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G9" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F10" t="s">
+        <v>118</v>
+      </c>
+      <c r="H10" t="s">
         <v>121</v>
-      </c>
-      <c r="B10" t="s">
-        <v>122</v>
-      </c>
-      <c r="C10" t="s">
-        <v>123</v>
-      </c>
-      <c r="D10" t="s">
-        <v>121</v>
-      </c>
-      <c r="E10" t="s">
-        <v>124</v>
-      </c>
-      <c r="F10" t="s">
-        <v>122</v>
-      </c>
-      <c r="H10" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B11" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>214</v>
+        <v>254</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="E11" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="F11" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G11" t="s">
         <v>24</v>
@@ -2113,7 +2142,10 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A36817BF-F161-418A-9B8F-87A18459EBCD}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
@@ -2249,9 +2281,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B396063C-A3E8-4F0D-BBD3-83031D2833E6}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="1" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -2328,15 +2360,11 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6417C9C4-F4DF-4AC8-B50B-4BF5CA8F6EE6}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
-    <col min="3" max="3" width="27.85546875" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" customWidth="1"/>
-    <col min="7" max="7" width="23.7109375" customWidth="1"/>
+    <col min="1" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -2367,19 +2395,19 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B2" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F2" t="s">
         <v>38</v>
@@ -2390,22 +2418,22 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E3" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="F3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="G3" t="s">
         <v>24</v>
@@ -2413,91 +2441,91 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B4" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C4" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E4" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="F4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="G4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F5" t="s">
         <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>162</v>
       </c>
       <c r="C7" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D7" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="E7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="F7" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>30</v>
@@ -2505,19 +2533,19 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>210</v>
+        <v>261</v>
       </c>
       <c r="D8" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="E8" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F8" t="s">
         <v>38</v>
@@ -2528,22 +2556,22 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>265</v>
+        <v>247</v>
       </c>
       <c r="D9" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="E9" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G9" t="s">
         <v>24</v>
@@ -2551,22 +2579,22 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C10" t="s">
-        <v>221</v>
+        <v>262</v>
       </c>
       <c r="D10" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G10" t="s">
         <v>24</v>
@@ -2574,22 +2602,22 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="B11" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="C11" t="s">
-        <v>230</v>
+        <v>263</v>
       </c>
       <c r="D11" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="E11" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="F11" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="G11" t="s">
         <v>30</v>
@@ -2597,19 +2625,19 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>234</v>
+        <v>221</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="D12" t="s">
-        <v>234</v>
+        <v>221</v>
       </c>
       <c r="E12" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F12" t="s">
         <v>38</v>
@@ -2620,22 +2648,22 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>238</v>
+        <v>225</v>
       </c>
       <c r="B13" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="C13" t="s">
-        <v>239</v>
+        <v>264</v>
       </c>
       <c r="D13" t="s">
-        <v>238</v>
+        <v>225</v>
       </c>
       <c r="E13" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="F13" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="G13" t="s">
         <v>24</v>
@@ -2643,42 +2671,42 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="B14" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="C14" t="s">
-        <v>244</v>
+        <v>265</v>
       </c>
       <c r="D14" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="E14" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="F14" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H14" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D15" t="s">
-        <v>263</v>
+        <v>246</v>
       </c>
       <c r="E15" t="s">
-        <v>263</v>
+        <v>246</v>
       </c>
       <c r="F15" t="s">
         <v>38</v>
@@ -2696,15 +2724,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919936B4-B1A4-46D7-993E-F45D36458108}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="1" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -2735,42 +2759,42 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B2" t="s">
         <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="E2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F2" t="s">
         <v>38</v>
       </c>
       <c r="G2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D3" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="E3" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -2781,19 +2805,19 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>182</v>
+        <v>270</v>
       </c>
       <c r="D4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="E4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="F4" t="s">
         <v>38</v>
@@ -2804,22 +2828,22 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B5" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C5" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="D5" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E5" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="F5" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G5" t="s">
         <v>24</v>
@@ -2827,22 +2851,22 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E6" t="s">
         <v>185</v>
       </c>
-      <c r="C6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D6" t="s">
-        <v>189</v>
-      </c>
-      <c r="E6" t="s">
-        <v>191</v>
-      </c>
       <c r="F6" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G6" t="s">
         <v>24</v>
@@ -2850,68 +2874,68 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>192</v>
+        <v>269</v>
       </c>
       <c r="D7" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E7" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G7" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="B8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D8" t="s">
+        <v>189</v>
+      </c>
+      <c r="E8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" t="s">
         <v>98</v>
       </c>
-      <c r="C8" t="s">
-        <v>196</v>
-      </c>
-      <c r="D8" t="s">
-        <v>195</v>
-      </c>
-      <c r="E8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F8" t="s">
-        <v>101</v>
-      </c>
       <c r="G8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B9" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C9" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D9" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="E9" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="F9" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="G9" t="s">
         <v>30</v>
@@ -2919,22 +2943,22 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B10" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C10" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D10" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="E10" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="F10" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="G10" t="s">
         <v>24</v>
@@ -2942,91 +2966,91 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B11" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C11" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D11" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="E11" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="F11" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="G11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B12" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="C12" t="s">
-        <v>219</v>
+        <v>268</v>
       </c>
       <c r="D12" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="E12" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="F12" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="G12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>231</v>
+        <v>218</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>231</v>
+        <v>267</v>
       </c>
       <c r="D13" t="s">
-        <v>231</v>
+        <v>218</v>
       </c>
       <c r="E13" t="s">
-        <v>232</v>
+        <v>219</v>
       </c>
       <c r="F13" t="s">
         <v>38</v>
       </c>
       <c r="G13" t="s">
-        <v>233</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="D14" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="E14" t="s">
-        <v>235</v>
+        <v>222</v>
       </c>
       <c r="F14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G14" t="s">
         <v>24</v>
@@ -3034,62 +3058,62 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="C15" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="D15" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="E15" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="F15" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="H15" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="C16" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="D16" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="E16" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="F16" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="H16" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="B17" t="s">
-        <v>253</v>
+        <v>237</v>
       </c>
       <c r="C17" t="s">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="D17" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="E17" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="F17" t="s">
-        <v>253</v>
+        <v>237</v>
       </c>
       <c r="G17" t="s">
         <v>24</v>
@@ -3097,25 +3121,25 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="D18" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="E18" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="F18" t="s">
         <v>29</v>
       </c>
       <c r="G18" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -3127,15 +3151,11 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF27F01-F832-4718-B945-C43E22A8DD17}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.42578125" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" customWidth="1"/>
-    <col min="3" max="3" width="25.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="29.42578125" customWidth="1"/>
-    <col min="7" max="7" width="21.28515625" customWidth="1"/>
+    <col min="1" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -3166,25 +3186,25 @@
     </row>
     <row r="2" spans="1:12" s="2" customFormat="1">
       <c r="A2" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s">
-        <v>138</v>
+        <v>273</v>
       </c>
       <c r="D2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H2"/>
       <c r="I2"/>
@@ -3194,25 +3214,25 @@
     </row>
     <row r="3" spans="1:12" s="2" customFormat="1">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>136</v>
+        <v>272</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H3"/>
       <c r="I3"/>
@@ -3222,25 +3242,25 @@
     </row>
     <row r="4" spans="1:12" s="2" customFormat="1">
       <c r="A4" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H4"/>
       <c r="I4"/>
@@ -3250,91 +3270,94 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>276</v>
       </c>
       <c r="D5" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E5" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F5" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="G5" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C6" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D6" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="G6" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B7" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D7" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G7" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>216</v>
+        <v>208</v>
+      </c>
+      <c r="B8" t="s">
+        <v>275</v>
       </c>
       <c r="C8" t="s">
-        <v>216</v>
+        <v>274</v>
       </c>
       <c r="D8" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="E8" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="F8" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed some errors, added opamp
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F550F98-AFBD-48A5-A977-80A112E7B8A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94AE6D52-B13C-445E-A712-71D6CCE3CE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="288">
   <si>
     <t>Part Number</t>
   </si>
@@ -910,6 +910,43 @@
   </si>
   <si>
     <t>LM239DR 14-SOIC</t>
+  </si>
+  <si>
+    <r>
+      <t>TL072</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Inter"/>
+      </rPr>
+      <t>ACDT</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>TL072</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Inter"/>
+      </rPr>
+      <t>ACDT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> SOIC-8</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -970,11 +1007,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Accent 3 2" xfId="1" xr:uid="{07D6D35A-A25D-4183-ACA2-756DA14CBAEA}"/>
@@ -2409,7 +2447,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6417C9C4-F4DF-4AC8-B50B-4BF5CA8F6EE6}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.85546875" customWidth="1"/>
@@ -2763,6 +2801,29 @@
       </c>
       <c r="G15" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F16" t="s">
+        <v>38</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BEEEEEP and analog revision
</commit_message>
<xml_diff>
--- a/library/analog.xlsx
+++ b/library/analog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{788B0DE9-D3C6-4FD5-8B71-ACE2572FE89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{376D85B2-949B-416F-A84A-C8A5A597BE2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="ADC" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,9 @@
     <sheet name="GPS" sheetId="5" r:id="rId5"/>
     <sheet name="GSM" sheetId="9" r:id="rId6"/>
     <sheet name="OPAMP" sheetId="6" r:id="rId7"/>
-    <sheet name="Other" sheetId="7" r:id="rId8"/>
+    <sheet name="MUX" sheetId="10" r:id="rId8"/>
     <sheet name="Sensor" sheetId="8" r:id="rId9"/>
+    <sheet name="Other" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="298">
   <si>
     <t>Part Number</t>
   </si>
@@ -885,15 +886,6 @@
     <t>AD5160BRJZ5-RL7</t>
   </si>
   <si>
-    <t>SG2525AP013TR</t>
-  </si>
-  <si>
-    <t>SG2525A</t>
-  </si>
-  <si>
-    <t>SG2525AP013TR 16-SOIC</t>
-  </si>
-  <si>
     <t>CD4066BM96</t>
   </si>
   <si>
@@ -916,15 +908,6 @@
   </si>
   <si>
     <t>TL072IDT SOIC-8</t>
-  </si>
-  <si>
-    <t>UC2825DWTR</t>
-  </si>
-  <si>
-    <t>UC2825</t>
-  </si>
-  <si>
-    <t>UC2825DWTR 16-SOIC (W)</t>
   </si>
   <si>
     <t>LM124DR</t>
@@ -1030,12 +1013,21 @@
       <t xml:space="preserve"> SOT23-5</t>
     </r>
   </si>
+  <si>
+    <t>ADG442BRZ</t>
+  </si>
+  <si>
+    <t>ADG44(1/2)</t>
+  </si>
+  <si>
+    <t>ADG442BRZ SOIC-16</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1059,14 +1051,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
@@ -1100,12 +1084,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Accent 3 2" xfId="1" xr:uid="{07D6D35A-A25D-4183-ACA2-756DA14CBAEA}"/>
@@ -1668,6 +1650,348 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919936B4-B1A4-46D7-993E-F45D36458108}">
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.140625" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" customWidth="1"/>
+    <col min="4" max="8" width="20.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="s">
+        <v>269</v>
+      </c>
+      <c r="D4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E4" t="s">
+        <v>177</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" t="s">
+        <v>178</v>
+      </c>
+      <c r="E5" t="s">
+        <v>181</v>
+      </c>
+      <c r="F5" t="s">
+        <v>182</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E6" t="s">
+        <v>185</v>
+      </c>
+      <c r="F6" t="s">
+        <v>182</v>
+      </c>
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>268</v>
+      </c>
+      <c r="D7" t="s">
+        <v>186</v>
+      </c>
+      <c r="E7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D8" t="s">
+        <v>189</v>
+      </c>
+      <c r="E8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B9" t="s">
+        <v>193</v>
+      </c>
+      <c r="C9" t="s">
+        <v>194</v>
+      </c>
+      <c r="D9" t="s">
+        <v>192</v>
+      </c>
+      <c r="E9" t="s">
+        <v>192</v>
+      </c>
+      <c r="F9" t="s">
+        <v>193</v>
+      </c>
+      <c r="G9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" t="s">
+        <v>199</v>
+      </c>
+      <c r="E10" t="s">
+        <v>199</v>
+      </c>
+      <c r="F10" t="s">
+        <v>198</v>
+      </c>
+      <c r="G10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C11" t="s">
+        <v>267</v>
+      </c>
+      <c r="D11" t="s">
+        <v>211</v>
+      </c>
+      <c r="E11" t="s">
+        <v>210</v>
+      </c>
+      <c r="F11" t="s">
+        <v>198</v>
+      </c>
+      <c r="G11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>218</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D12" t="s">
+        <v>218</v>
+      </c>
+      <c r="E12" t="s">
+        <v>219</v>
+      </c>
+      <c r="F12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>223</v>
+      </c>
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
+        <v>224</v>
+      </c>
+      <c r="D13" t="s">
+        <v>223</v>
+      </c>
+      <c r="E13" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>276</v>
+      </c>
+      <c r="B14" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" t="s">
+        <v>238</v>
+      </c>
+      <c r="D14" t="s">
+        <v>236</v>
+      </c>
+      <c r="E14" t="s">
+        <v>236</v>
+      </c>
+      <c r="F14" t="s">
+        <v>237</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E834B2D-3CFC-49B2-A2B4-67F2231F306F}">
   <dimension ref="A1:H7"/>
@@ -1849,7 +2173,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE4D8C3D-D832-496B-AB92-259D2AD291EC}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.85546875" customWidth="1"/>
@@ -1884,236 +2208,188 @@
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" t="s">
         <v>78</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="3"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="3" t="s">
+      <c r="A3" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>80</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>79</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" t="s">
         <v>81</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" t="s">
         <v>38</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="3" t="s">
+      <c r="A4" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" t="s">
         <v>84</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="3" t="s">
+      <c r="A5" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" t="s">
         <v>88</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" t="s">
         <v>89</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="3" t="s">
+      <c r="A6" t="s">
         <v>201</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s">
         <v>162</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" t="s">
         <v>202</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" t="s">
         <v>201</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" t="s">
         <v>88</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" t="s">
         <v>162</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" t="s">
         <v>116</v>
       </c>
-      <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>227</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s">
         <v>257</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" t="s">
         <v>258</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" t="s">
         <v>234</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" t="s">
         <v>259</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" t="s">
         <v>229</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3" t="s">
+      <c r="H7" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="B8" s="3" t="s">
+      <c r="A8" t="s">
+        <v>280</v>
+      </c>
+      <c r="B8" t="s">
         <v>158</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="C8" t="s">
+        <v>282</v>
+      </c>
+      <c r="D8" t="s">
+        <v>280</v>
+      </c>
+      <c r="E8" t="s">
+        <v>281</v>
+      </c>
+      <c r="F8" t="s">
         <v>158</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="3"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="B9" s="3" t="s">
+      <c r="A9" t="s">
+        <v>293</v>
+      </c>
+      <c r="B9" t="s">
         <v>162</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="F9" s="3" t="s">
+      <c r="C9" t="s">
+        <v>294</v>
+      </c>
+      <c r="D9" t="s">
+        <v>293</v>
+      </c>
+      <c r="E9" t="s">
+        <v>292</v>
+      </c>
+      <c r="F9" t="s">
         <v>162</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3011,16 +3287,16 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>149</v>
@@ -3037,16 +3313,16 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="2" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>156</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>153</v>
@@ -3063,16 +3339,16 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>149</v>
@@ -3130,13 +3406,17 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919936B4-B1A4-46D7-993E-F45D36458108}">
-  <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0E3ABE5-1DA9-4AF4-85F1-A7A6190653DE}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="20.85546875" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" customWidth="1"/>
-    <col min="4" max="8" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -3167,91 +3447,91 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>168</v>
+        <v>289</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>198</v>
       </c>
       <c r="C2" t="s">
-        <v>169</v>
+        <v>291</v>
       </c>
       <c r="D2" t="s">
-        <v>170</v>
+        <v>289</v>
       </c>
       <c r="E2" t="s">
-        <v>171</v>
+        <v>290</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>198</v>
       </c>
       <c r="G2" t="s">
-        <v>172</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>173</v>
+        <v>277</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>174</v>
+        <v>279</v>
       </c>
       <c r="D3" t="s">
-        <v>173</v>
+        <v>277</v>
       </c>
       <c r="E3" t="s">
-        <v>175</v>
+        <v>278</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>158</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>176</v>
+        <v>239</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D4" t="s">
-        <v>176</v>
+        <v>239</v>
       </c>
       <c r="E4" t="s">
-        <v>177</v>
+        <v>240</v>
       </c>
       <c r="F4" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>24</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="B5" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="C5" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="D5" t="s">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="E5" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="F5" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="G5" t="s">
         <v>24</v>
@@ -3259,419 +3539,50 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>183</v>
-      </c>
-      <c r="B6" t="s">
-        <v>179</v>
+        <v>231</v>
       </c>
       <c r="C6" t="s">
-        <v>184</v>
+        <v>231</v>
       </c>
       <c r="D6" t="s">
-        <v>183</v>
+        <v>231</v>
       </c>
       <c r="E6" t="s">
-        <v>185</v>
+        <v>231</v>
       </c>
       <c r="F6" t="s">
-        <v>182</v>
-      </c>
-      <c r="G6" t="s">
-        <v>24</v>
+        <v>232</v>
+      </c>
+      <c r="H6" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>295</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>196</v>
       </c>
       <c r="C7" t="s">
-        <v>268</v>
+        <v>297</v>
       </c>
       <c r="D7" t="s">
-        <v>186</v>
+        <v>295</v>
       </c>
       <c r="E7" t="s">
-        <v>187</v>
+        <v>296</v>
       </c>
       <c r="F7" t="s">
-        <v>50</v>
+        <v>198</v>
       </c>
       <c r="G7" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>189</v>
-      </c>
-      <c r="B8" t="s">
-        <v>95</v>
-      </c>
-      <c r="C8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D8" t="s">
-        <v>189</v>
-      </c>
-      <c r="E8" t="s">
-        <v>191</v>
-      </c>
-      <c r="F8" t="s">
-        <v>98</v>
-      </c>
-      <c r="G8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>192</v>
-      </c>
-      <c r="B9" t="s">
-        <v>193</v>
-      </c>
-      <c r="C9" t="s">
-        <v>194</v>
-      </c>
-      <c r="D9" t="s">
-        <v>192</v>
-      </c>
-      <c r="E9" t="s">
-        <v>192</v>
-      </c>
-      <c r="F9" t="s">
-        <v>193</v>
-      </c>
-      <c r="G9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>195</v>
-      </c>
-      <c r="B10" t="s">
-        <v>196</v>
-      </c>
-      <c r="C10" t="s">
-        <v>197</v>
-      </c>
-      <c r="D10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E10" t="s">
-        <v>195</v>
-      </c>
-      <c r="F10" t="s">
-        <v>198</v>
-      </c>
-      <c r="G10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>199</v>
-      </c>
-      <c r="B11" t="s">
-        <v>196</v>
-      </c>
-      <c r="C11" t="s">
-        <v>200</v>
-      </c>
-      <c r="D11" t="s">
-        <v>199</v>
-      </c>
-      <c r="E11" t="s">
-        <v>199</v>
-      </c>
-      <c r="F11" t="s">
-        <v>198</v>
-      </c>
-      <c r="G11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>211</v>
-      </c>
-      <c r="B12" t="s">
-        <v>196</v>
-      </c>
-      <c r="C12" t="s">
-        <v>267</v>
-      </c>
-      <c r="D12" t="s">
-        <v>211</v>
-      </c>
-      <c r="E12" t="s">
-        <v>210</v>
-      </c>
-      <c r="F12" t="s">
-        <v>198</v>
-      </c>
-      <c r="G12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>218</v>
-      </c>
-      <c r="B13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" t="s">
-        <v>266</v>
-      </c>
-      <c r="D13" t="s">
-        <v>218</v>
-      </c>
-      <c r="E13" t="s">
-        <v>219</v>
-      </c>
-      <c r="F13" t="s">
-        <v>38</v>
-      </c>
-      <c r="G13" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>223</v>
-      </c>
-      <c r="B14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" t="s">
-        <v>224</v>
-      </c>
-      <c r="D14" t="s">
-        <v>223</v>
-      </c>
-      <c r="E14" t="s">
-        <v>222</v>
-      </c>
-      <c r="F14" t="s">
-        <v>50</v>
-      </c>
-      <c r="G14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>231</v>
-      </c>
-      <c r="C15" t="s">
-        <v>231</v>
-      </c>
-      <c r="D15" t="s">
-        <v>231</v>
-      </c>
-      <c r="E15" t="s">
-        <v>231</v>
-      </c>
-      <c r="F15" t="s">
-        <v>232</v>
-      </c>
-      <c r="H15" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>232</v>
-      </c>
-      <c r="C16" t="s">
-        <v>232</v>
-      </c>
-      <c r="D16" t="s">
-        <v>232</v>
-      </c>
-      <c r="E16" t="s">
-        <v>232</v>
-      </c>
-      <c r="F16" t="s">
-        <v>232</v>
-      </c>
-      <c r="H16" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>276</v>
-      </c>
-      <c r="B17" t="s">
-        <v>237</v>
-      </c>
-      <c r="C17" t="s">
-        <v>238</v>
-      </c>
-      <c r="D17" t="s">
-        <v>236</v>
-      </c>
-      <c r="E17" t="s">
-        <v>236</v>
-      </c>
-      <c r="F17" t="s">
-        <v>237</v>
-      </c>
-      <c r="G17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>